<commit_message>
rate of production and destruction analysis now possible again from GUI
A new module is included and functioning for rate of production and destruction analysis (change tendencies) and can be called from the PyCHAM GUI
</commit_message>
<xml_diff>
--- a/PyCHAM/output/Myanmar_NOCs_paper_Zhang_etal/Myanmar_results/results_summary.xlsx
+++ b/PyCHAM/output/Myanmar_NOCs_paper_Zhang_etal/Myanmar_results/results_summary.xlsx
@@ -8,19 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://livemanchesterac-my.sharepoint.com/personal/simon_omeara_manchester_ac_uk/Documents/GitHub/PyCHAM/PyCHAM/output/Myanmar_NOCs_paper_Zhang_etal/Myanmar_results_summary/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="214" documentId="8_{E8B0B34E-3CE5-C34E-8A2F-7DC02E83A91F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9F32DD5-81F1-7446-916E-0DD403625E20}"/>
+  <xr:revisionPtr revIDLastSave="223" documentId="8_{E8B0B34E-3CE5-C34E-8A2F-7DC02E83A91F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB034ADE-1D76-D74D-B87A-C8079987296D}"/>
   <bookViews>
     <workbookView xWindow="320" yWindow="4560" windowWidth="31040" windowHeight="15900" xr2:uid="{0F592B18-6E21-ED45-9530-91214C8428D9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">Sheet1!$O$2:$O$7</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">Sheet1!$O$2:$O$7</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">Sheet1!$O$2:$O$7</definedName>
-  </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="29">
   <si>
     <t>RH (%)</t>
   </si>
@@ -119,6 +114,15 @@
   </si>
   <si>
     <t>particle-phase C8/C6 ratio w/o varying HONO influx rate (no HONO dependence on gas-phase water concentration test, influx rate constant at 0.00066 ppb/s)</t>
+  </si>
+  <si>
+    <t>Season</t>
+  </si>
+  <si>
+    <t>Summer</t>
+  </si>
+  <si>
+    <t>Winter</t>
   </si>
 </sst>
 </file>
@@ -302,7 +306,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$D$2:$D$8</c:f>
+              <c:f>Sheet1!$E$2:$E$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -329,7 +333,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$O$2:$O$8</c:f>
+              <c:f>Sheet1!$P$2:$P$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -391,7 +395,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$D$2:$D$4</c:f>
+              <c:f>Sheet1!$E$2:$E$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -409,7 +413,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$P$2:$P$4</c:f>
+              <c:f>Sheet1!$Q$2:$Q$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -1320,16 +1324,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>565150</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>101600</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>317500</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1355,6 +1359,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1674,10 +1682,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0B6F0C6-453A-A44C-9FB0-014D66AD5BD2}">
-  <dimension ref="A1:S16"/>
+  <dimension ref="A1:T16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -1685,495 +1693,516 @@
         <v>14</v>
       </c>
       <c r="C1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" t="s">
         <v>16</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>0</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>19</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>18</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>2</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>1</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>5</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>6</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>7</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="Q1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="Q1" s="4"/>
-      <c r="R1" t="s">
+      <c r="R1" s="4"/>
+      <c r="S1" t="s">
         <v>21</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>15</v>
       </c>
       <c r="B2">
         <v>302.95</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2">
         <v>90</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>40</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>3</v>
       </c>
-      <c r="F2" s="2">
+      <c r="G2" s="2">
         <v>5200000</v>
       </c>
-      <c r="G2" s="2">
+      <c r="H2" s="2">
         <v>27.97</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>3.57</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>0.4</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>0.26</v>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>0.37</v>
       </c>
-      <c r="L2">
+      <c r="M2">
         <v>0.39</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>14.72</v>
       </c>
-      <c r="N2">
+      <c r="O2">
         <v>6.28</v>
       </c>
-      <c r="O2" s="3">
-        <f>N2/M2</f>
+      <c r="P2" s="3">
+        <f>O2/N2</f>
         <v>0.4266304347826087</v>
       </c>
-      <c r="P2">
+      <c r="Q2">
         <v>0.27</v>
       </c>
-      <c r="R2">
+      <c r="S2">
         <f>(7.23/26.1)</f>
         <v>0.27701149425287358</v>
       </c>
-      <c r="S2">
+      <c r="T2">
         <f>(6.28/14.72)</f>
         <v>0.4266304347826087</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>15</v>
       </c>
       <c r="B3">
         <v>295.5</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3">
         <v>1</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>60</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>3</v>
       </c>
-      <c r="F3" s="2">
+      <c r="G3" s="2">
         <v>3400000</v>
       </c>
-      <c r="G3" s="2">
+      <c r="H3" s="2">
         <v>48.48</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>3.58</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>0.41</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>0.27</v>
       </c>
-      <c r="K3">
+      <c r="L3">
         <v>0.39</v>
       </c>
-      <c r="L3">
+      <c r="M3">
         <v>0.4</v>
       </c>
-      <c r="M3">
+      <c r="N3">
         <v>6.27</v>
       </c>
-      <c r="N3">
+      <c r="O3">
         <v>3.4</v>
       </c>
-      <c r="O3" s="3">
-        <f t="shared" ref="O3:O4" si="0">N3/M3</f>
+      <c r="P3" s="3">
+        <f t="shared" ref="P3:P4" si="0">O3/N3</f>
         <v>0.54226475279106856</v>
       </c>
-      <c r="P3">
+      <c r="Q3">
         <v>0.48</v>
       </c>
-      <c r="R3">
+      <c r="S3">
         <f>(3.93/8.59)</f>
         <v>0.45750873108265427</v>
       </c>
-      <c r="S3">
+      <c r="T3">
         <f>(3.4/6.27)</f>
         <v>0.54226475279106856</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>15</v>
       </c>
       <c r="B4">
         <v>295.5</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4">
         <v>1</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>80</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>3</v>
       </c>
-      <c r="F4" s="2">
+      <c r="G4" s="2">
         <v>3700000</v>
       </c>
-      <c r="G4" s="2">
+      <c r="H4" s="2">
         <v>116.06</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>3.58</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>0.41</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>0.27</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>0.39</v>
       </c>
-      <c r="L4">
+      <c r="M4">
         <v>0.4</v>
       </c>
-      <c r="M4">
+      <c r="N4">
         <v>7.01</v>
       </c>
-      <c r="N4">
+      <c r="O4">
         <v>4.8600000000000003</v>
       </c>
-      <c r="O4" s="3">
+      <c r="P4" s="3">
         <f t="shared" si="0"/>
         <v>0.69329529243937238</v>
       </c>
-      <c r="P4">
+      <c r="Q4">
         <v>0.57999999999999996</v>
       </c>
-      <c r="R4">
+      <c r="S4">
         <f>(6.04/10.72)</f>
         <v>0.56343283582089554</v>
       </c>
-      <c r="S4">
+      <c r="T4">
         <f>(4.86/7.01)</f>
         <v>0.69329529243937238</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="O5" s="3"/>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="P5" s="3"/>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>17</v>
       </c>
       <c r="B6">
         <v>303.55</v>
       </c>
-      <c r="C6">
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6">
         <v>90</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>70</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>1</v>
       </c>
-      <c r="F6" s="2">
+      <c r="G6" s="2">
         <v>7700000</v>
       </c>
-      <c r="G6" s="2">
+      <c r="H6" s="2">
         <v>38.159999999999997</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>1.19</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>0.4</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>0.25</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <v>0.36</v>
       </c>
-      <c r="L6">
+      <c r="M6">
         <v>0.38</v>
       </c>
-      <c r="M6">
+      <c r="N6">
         <v>8.7100000000000009</v>
       </c>
-      <c r="N6">
+      <c r="O6">
         <v>5.0599999999999996</v>
       </c>
-      <c r="O6" s="3">
-        <f>N6/M6</f>
+      <c r="P6" s="3">
+        <f>O6/N6</f>
         <v>0.58094144661308833</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>17</v>
       </c>
       <c r="B7">
         <v>300.55</v>
       </c>
-      <c r="C7">
+      <c r="C7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7">
         <v>1</v>
       </c>
-      <c r="D7">
+      <c r="E7">
         <v>70</v>
       </c>
-      <c r="E7">
+      <c r="F7">
         <v>2</v>
       </c>
-      <c r="F7" s="2">
+      <c r="G7" s="2">
         <v>4900000</v>
       </c>
-      <c r="G7" s="2">
+      <c r="H7" s="2">
         <v>48.15</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>2.38</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <v>0.4</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>0.26</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>0.38</v>
       </c>
-      <c r="L7">
+      <c r="M7">
         <v>0.39</v>
       </c>
-      <c r="M7">
+      <c r="N7">
         <v>8.06</v>
       </c>
-      <c r="N7">
+      <c r="O7">
         <v>4.18</v>
       </c>
-      <c r="O7" s="3">
-        <f>N7/M7</f>
+      <c r="P7" s="3">
+        <f>O7/N7</f>
         <v>0.51861042183622819</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>20</v>
       </c>
       <c r="B8">
         <v>300.55</v>
       </c>
-      <c r="C8">
+      <c r="C8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8">
         <v>1</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>70</v>
       </c>
-      <c r="E8">
+      <c r="F8">
         <v>1</v>
       </c>
-      <c r="F8" s="2">
+      <c r="G8" s="2">
         <v>5100000</v>
       </c>
-      <c r="G8" s="2">
+      <c r="H8" s="2">
         <v>48.23</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <v>1.19</v>
       </c>
-      <c r="I8">
+      <c r="J8">
         <v>0.4</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>0.26</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <v>0.38</v>
       </c>
-      <c r="L8">
+      <c r="M8">
         <v>0.39</v>
       </c>
-      <c r="M8">
+      <c r="N8">
         <v>4.42</v>
       </c>
-      <c r="N8">
+      <c r="O8">
         <v>4.43</v>
       </c>
-      <c r="O8" s="3">
-        <f>N8/M8</f>
+      <c r="P8" s="3">
+        <f>O8/N8</f>
         <v>1.002262443438914</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="H9" t="s">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="I9" t="s">
         <v>8</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>9</v>
       </c>
-      <c r="J9" t="s">
+      <c r="K9" t="s">
         <v>10</v>
       </c>
-      <c r="K9" s="1" t="s">
+      <c r="L9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="L9" s="1" t="s">
+      <c r="M9" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="H10">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="I10">
         <v>11.22</v>
       </c>
-      <c r="I10">
+      <c r="J10">
         <v>1.72</v>
       </c>
-      <c r="J10">
+      <c r="K10">
         <v>1.1100000000000001</v>
       </c>
-      <c r="K10">
+      <c r="L10">
         <v>1.59</v>
       </c>
-      <c r="L10">
+      <c r="M10">
         <v>1.65</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="H11">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="I11">
         <v>11.53</v>
       </c>
-      <c r="I11">
+      <c r="J11">
         <v>1.79</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <v>1.17</v>
       </c>
-      <c r="K11">
+      <c r="L11">
         <v>1.7</v>
       </c>
-      <c r="L11">
+      <c r="M11">
         <v>1.75</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="H12">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="I12">
         <v>11.53</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <v>1.79</v>
       </c>
-      <c r="J12">
+      <c r="K12">
         <v>1.1599999999999999</v>
       </c>
-      <c r="K12">
+      <c r="L12">
         <v>1.7</v>
       </c>
-      <c r="L12">
+      <c r="M12">
         <v>1.74</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="H14">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="I14">
         <v>3.72</v>
       </c>
-      <c r="I14">
+      <c r="J14">
         <v>1.68</v>
       </c>
-      <c r="J14">
+      <c r="K14">
         <v>1.07</v>
       </c>
-      <c r="K14">
+      <c r="L14">
         <v>1.52</v>
       </c>
-      <c r="L14">
+      <c r="M14">
         <v>1.6</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="H15">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="I15">
         <v>7.55</v>
       </c>
-      <c r="I15">
+      <c r="J15">
         <v>1.74</v>
       </c>
-      <c r="J15">
+      <c r="K15">
         <v>1.1200000000000001</v>
       </c>
-      <c r="K15">
+      <c r="L15">
         <v>1.62</v>
       </c>
-      <c r="L15">
+      <c r="M15">
         <v>1.68</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="H16">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="I16">
         <v>3.77</v>
       </c>
-      <c r="I16">
+      <c r="J16">
         <v>1.74</v>
       </c>
-      <c r="J16">
+      <c r="K16">
         <v>1.1200000000000001</v>
       </c>
-      <c r="K16">
+      <c r="L16">
         <v>1.62</v>
       </c>
-      <c r="L16">
+      <c r="M16">
         <v>1.68</v>
       </c>
     </row>

</xml_diff>